<commit_message>
Fix Service Worker interference with Vite HMR and Google Fonts
</commit_message>
<xml_diff>
--- a/backend/data/users_export.xlsx
+++ b/backend/data/users_export.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -570,13 +570,13 @@
         <v>p003</v>
       </c>
       <c r="B7" t="str">
-        <v>Realtime User</v>
+        <v>Nafis Shaikh</v>
       </c>
       <c r="C7" t="str">
         <v>passenger</v>
       </c>
       <c r="D7" t="str">
-        <v>realuser49744@gmail.com</v>
+        <v>nafisabidshaikh143@gmail.com</v>
       </c>
       <c r="E7" t="str">
         <v>MPC-7003</v>
@@ -588,7 +588,7 @@
         <v>(encrypted - set during signup)</v>
       </c>
       <c r="H7" t="str">
-        <v>realuser49744@gmail.com</v>
+        <v>nafisabidshaikh143@gmail.com</v>
       </c>
     </row>
     <row r="8">
@@ -596,13 +596,13 @@
         <v>p004</v>
       </c>
       <c r="B8" t="str">
-        <v>Persist One</v>
+        <v>Nafis Shaikh</v>
       </c>
       <c r="C8" t="str">
         <v>passenger</v>
       </c>
       <c r="D8" t="str">
-        <v>persist78192@gmail.com</v>
+        <v>nafisabidshaikh@gmail.com</v>
       </c>
       <c r="E8" t="str">
         <v>MPC-7004</v>
@@ -614,7 +614,7 @@
         <v>(encrypted - set during signup)</v>
       </c>
       <c r="H8" t="str">
-        <v>persist78192@gmail.com</v>
+        <v>nafisabidshaikh@gmail.com</v>
       </c>
     </row>
     <row r="9">
@@ -622,13 +622,13 @@
         <v>p005</v>
       </c>
       <c r="B9" t="str">
-        <v>Persist Two</v>
+        <v>AARISH KHAN</v>
       </c>
       <c r="C9" t="str">
         <v>passenger</v>
       </c>
       <c r="D9" t="str">
-        <v>persist75743@gmail.com</v>
+        <v>aarishkhan@theeemcoe.org</v>
       </c>
       <c r="E9" t="str">
         <v>MPC-7005</v>
@@ -640,38 +640,12 @@
         <v>(encrypted - set during signup)</v>
       </c>
       <c r="H9" t="str">
-        <v>persist75743@gmail.com</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>p006</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Nafis Shaikh</v>
-      </c>
-      <c r="C10" t="str">
-        <v>passenger</v>
-      </c>
-      <c r="D10" t="str">
-        <v>nafisabidshaikh12@gmail.com</v>
-      </c>
-      <c r="E10" t="str">
-        <v>MPC-7006</v>
-      </c>
-      <c r="F10" t="str">
-        <v>—</v>
-      </c>
-      <c r="G10" t="str">
-        <v>(encrypted - set during signup)</v>
-      </c>
-      <c r="H10" t="str">
-        <v>nafisabidshaikh12@gmail.com</v>
+        <v>aarishkhan@theeemcoe.org</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add schedule management features: create, update, delete, and fetch schedules
</commit_message>
<xml_diff>
--- a/backend/data/users_export.xlsx
+++ b/backend/data/users_export.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -429,7 +429,7 @@
         <v>Department</v>
       </c>
       <c r="G1" t="str">
-        <v>Password (Plain)</v>
+        <v>Password Storage</v>
       </c>
       <c r="H1" t="str">
         <v>Login Identifier</v>
@@ -455,7 +455,7 @@
         <v>Administration</v>
       </c>
       <c r="G2" t="str">
-        <v>Admin@1234</v>
+        <v>Hashed (scrypt + salt)</v>
       </c>
       <c r="H2" t="str">
         <v>MRS-A-001</v>
@@ -481,7 +481,7 @@
         <v>Operations</v>
       </c>
       <c r="G3" t="str">
-        <v>Super@1234</v>
+        <v>Hashed (scrypt + salt)</v>
       </c>
       <c r="H3" t="str">
         <v>MRS-S-042</v>
@@ -507,7 +507,7 @@
         <v>Station Management</v>
       </c>
       <c r="G4" t="str">
-        <v>Empl@1234</v>
+        <v>Hashed (scrypt + salt)</v>
       </c>
       <c r="H4" t="str">
         <v>MRS-E-187</v>
@@ -515,94 +515,94 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>p001</v>
+        <v>p003</v>
       </c>
       <c r="B5" t="str">
-        <v>Rahul Mishra</v>
+        <v>Nafis Shaikh</v>
       </c>
       <c r="C5" t="str">
         <v>passenger</v>
       </c>
       <c r="D5" t="str">
-        <v>user001</v>
+        <v>nafisabidshaikh143@gmail.com</v>
       </c>
       <c r="E5" t="str">
-        <v>MPC-7842</v>
+        <v>MPC-7003</v>
       </c>
       <c r="F5" t="str">
         <v>—</v>
       </c>
       <c r="G5" t="str">
-        <v>pass123</v>
+        <v>Hashed (scrypt + salt)</v>
       </c>
       <c r="H5" t="str">
-        <v>user001</v>
+        <v>nafisabidshaikh143@gmail.com</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>p002</v>
+        <v>p004</v>
       </c>
       <c r="B6" t="str">
-        <v>Ananya Singh</v>
+        <v>Nafis Shaikh</v>
       </c>
       <c r="C6" t="str">
         <v>passenger</v>
       </c>
       <c r="D6" t="str">
-        <v>user002</v>
+        <v>nafisabidshaikh12@gmail.com</v>
       </c>
       <c r="E6" t="str">
-        <v>MPC-3391</v>
+        <v>MPC-7004</v>
       </c>
       <c r="F6" t="str">
         <v>—</v>
       </c>
       <c r="G6" t="str">
-        <v>metro2024</v>
+        <v>Hashed (scrypt + salt)</v>
       </c>
       <c r="H6" t="str">
-        <v>user002</v>
+        <v>nafisabidshaikh12@gmail.com</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>p003</v>
+        <v>p005</v>
       </c>
       <c r="B7" t="str">
-        <v>Nafis Shaikh</v>
+        <v>AARISH KHAN</v>
       </c>
       <c r="C7" t="str">
         <v>passenger</v>
       </c>
       <c r="D7" t="str">
-        <v>nafisabidshaikh143@gmail.com</v>
+        <v>aarishkhan@theeemcoe.org</v>
       </c>
       <c r="E7" t="str">
-        <v>MPC-7003</v>
+        <v>MPC-7005</v>
       </c>
       <c r="F7" t="str">
         <v>—</v>
       </c>
       <c r="G7" t="str">
-        <v>(encrypted - set during signup)</v>
+        <v>Hashed (scrypt + salt)</v>
       </c>
       <c r="H7" t="str">
-        <v>nafisabidshaikh143@gmail.com</v>
+        <v>aarishkhan@theeemcoe.org</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>p004</v>
+        <v>p006</v>
       </c>
       <c r="B8" t="str">
-        <v>Nafis Shaikh</v>
+        <v>Test Passenger</v>
       </c>
       <c r="C8" t="str">
         <v>passenger</v>
       </c>
       <c r="D8" t="str">
-        <v>nafisabidshaikh@gmail.com</v>
+        <v>testuser3860</v>
       </c>
       <c r="E8" t="str">
         <v>MPC-7004</v>
@@ -611,41 +611,15 @@
         <v>—</v>
       </c>
       <c r="G8" t="str">
-        <v>(encrypted - set during signup)</v>
+        <v>Hashed (scrypt + salt)</v>
       </c>
       <c r="H8" t="str">
-        <v>nafisabidshaikh@gmail.com</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>p005</v>
-      </c>
-      <c r="B9" t="str">
-        <v>AARISH KHAN</v>
-      </c>
-      <c r="C9" t="str">
-        <v>passenger</v>
-      </c>
-      <c r="D9" t="str">
-        <v>aarishkhan@theeemcoe.org</v>
-      </c>
-      <c r="E9" t="str">
-        <v>MPC-7005</v>
-      </c>
-      <c r="F9" t="str">
-        <v>—</v>
-      </c>
-      <c r="G9" t="str">
-        <v>(encrypted - set during signup)</v>
-      </c>
-      <c r="H9" t="str">
-        <v>aarishkhan@theeemcoe.org</v>
+        <v>testuser3860</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor schedule management: update API integration, enhance schedule creation, and improve data handling
</commit_message>
<xml_diff>
--- a/backend/data/users_export.xlsx
+++ b/backend/data/users_export.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -429,7 +429,7 @@
         <v>Department</v>
       </c>
       <c r="G1" t="str">
-        <v>Password (Plain)</v>
+        <v>Password Storage</v>
       </c>
       <c r="H1" t="str">
         <v>Login Identifier</v>
@@ -455,7 +455,7 @@
         <v>Administration</v>
       </c>
       <c r="G2" t="str">
-        <v>Admin@1234</v>
+        <v>Hashed (scrypt + salt)</v>
       </c>
       <c r="H2" t="str">
         <v>MRS-A-001</v>
@@ -481,7 +481,7 @@
         <v>Operations</v>
       </c>
       <c r="G3" t="str">
-        <v>Super@1234</v>
+        <v>Hashed (scrypt + salt)</v>
       </c>
       <c r="H3" t="str">
         <v>MRS-S-042</v>
@@ -507,7 +507,7 @@
         <v>Station Management</v>
       </c>
       <c r="G4" t="str">
-        <v>Empl@1234</v>
+        <v>Hashed (scrypt + salt)</v>
       </c>
       <c r="H4" t="str">
         <v>MRS-E-187</v>
@@ -515,94 +515,94 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>p001</v>
+        <v>p003</v>
       </c>
       <c r="B5" t="str">
-        <v>Rahul Mishra</v>
+        <v>Nafis Shaikh</v>
       </c>
       <c r="C5" t="str">
         <v>passenger</v>
       </c>
       <c r="D5" t="str">
-        <v>user001</v>
+        <v>nafisabidshaikh143@gmail.com</v>
       </c>
       <c r="E5" t="str">
-        <v>MPC-7842</v>
+        <v>MPC-7003</v>
       </c>
       <c r="F5" t="str">
         <v>—</v>
       </c>
       <c r="G5" t="str">
-        <v>pass123</v>
+        <v>Hashed (scrypt + salt)</v>
       </c>
       <c r="H5" t="str">
-        <v>user001</v>
+        <v>nafisabidshaikh143@gmail.com</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>p002</v>
+        <v>p004</v>
       </c>
       <c r="B6" t="str">
-        <v>Ananya Singh</v>
+        <v>Nafis Shaikh</v>
       </c>
       <c r="C6" t="str">
         <v>passenger</v>
       </c>
       <c r="D6" t="str">
-        <v>user002</v>
+        <v>nafisabidshaikh12@gmail.com</v>
       </c>
       <c r="E6" t="str">
-        <v>MPC-3391</v>
+        <v>MPC-7004</v>
       </c>
       <c r="F6" t="str">
         <v>—</v>
       </c>
       <c r="G6" t="str">
-        <v>metro2024</v>
+        <v>Hashed (scrypt + salt)</v>
       </c>
       <c r="H6" t="str">
-        <v>user002</v>
+        <v>nafisabidshaikh12@gmail.com</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>p003</v>
+        <v>p005</v>
       </c>
       <c r="B7" t="str">
-        <v>Nafis Shaikh</v>
+        <v>AARISH KHAN</v>
       </c>
       <c r="C7" t="str">
         <v>passenger</v>
       </c>
       <c r="D7" t="str">
-        <v>nafisabidshaikh143@gmail.com</v>
+        <v>aarishkhan@theeemcoe.org</v>
       </c>
       <c r="E7" t="str">
-        <v>MPC-7003</v>
+        <v>MPC-7005</v>
       </c>
       <c r="F7" t="str">
         <v>—</v>
       </c>
       <c r="G7" t="str">
-        <v>(encrypted - set during signup)</v>
+        <v>Hashed (scrypt + salt)</v>
       </c>
       <c r="H7" t="str">
-        <v>nafisabidshaikh143@gmail.com</v>
+        <v>aarishkhan@theeemcoe.org</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>p004</v>
+        <v>p006</v>
       </c>
       <c r="B8" t="str">
-        <v>Nafis Shaikh</v>
+        <v>Test Passenger</v>
       </c>
       <c r="C8" t="str">
         <v>passenger</v>
       </c>
       <c r="D8" t="str">
-        <v>nafisabidshaikh@gmail.com</v>
+        <v>testuser3860</v>
       </c>
       <c r="E8" t="str">
         <v>MPC-7004</v>
@@ -611,41 +611,15 @@
         <v>—</v>
       </c>
       <c r="G8" t="str">
-        <v>(encrypted - set during signup)</v>
+        <v>Hashed (scrypt + salt)</v>
       </c>
       <c r="H8" t="str">
-        <v>nafisabidshaikh@gmail.com</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>p005</v>
-      </c>
-      <c r="B9" t="str">
-        <v>AARISH KHAN</v>
-      </c>
-      <c r="C9" t="str">
-        <v>passenger</v>
-      </c>
-      <c r="D9" t="str">
-        <v>aarishkhan@theeemcoe.org</v>
-      </c>
-      <c r="E9" t="str">
-        <v>MPC-7005</v>
-      </c>
-      <c r="F9" t="str">
-        <v>—</v>
-      </c>
-      <c r="G9" t="str">
-        <v>(encrypted - set during signup)</v>
-      </c>
-      <c r="H9" t="str">
-        <v>aarishkhan@theeemcoe.org</v>
+        <v>testuser3860</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement dashboard UI with role-based navigation, station metrics, and backend integration
</commit_message>
<xml_diff>
--- a/backend/data/users_export.xlsx
+++ b/backend/data/users_export.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -617,9 +617,35 @@
         <v>testuser3860</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>p007</v>
+      </c>
+      <c r="B9" t="str">
+        <v>API Tester</v>
+      </c>
+      <c r="C9" t="str">
+        <v>passenger</v>
+      </c>
+      <c r="D9" t="str">
+        <v>testuser2782</v>
+      </c>
+      <c r="E9" t="str">
+        <v>MPC-7005</v>
+      </c>
+      <c r="F9" t="str">
+        <v>—</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Hashed (scrypt + salt)</v>
+      </c>
+      <c r="H9" t="str">
+        <v>testuser2782</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: initialize sample metro rail schedules and user account data store
</commit_message>
<xml_diff>
--- a/backend/data/users_export.xlsx
+++ b/backend/data/users_export.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H12"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -617,9 +617,113 @@
         <v>testuser3860</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>p007</v>
+      </c>
+      <c r="B9" t="str">
+        <v>API Tester</v>
+      </c>
+      <c r="C9" t="str">
+        <v>passenger</v>
+      </c>
+      <c r="D9" t="str">
+        <v>testuser832</v>
+      </c>
+      <c r="E9" t="str">
+        <v>MPC-7005</v>
+      </c>
+      <c r="F9" t="str">
+        <v>—</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Hashed (scrypt + salt)</v>
+      </c>
+      <c r="H9" t="str">
+        <v>testuser832</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>p008</v>
+      </c>
+      <c r="B10" t="str">
+        <v>API Tester</v>
+      </c>
+      <c r="C10" t="str">
+        <v>passenger</v>
+      </c>
+      <c r="D10" t="str">
+        <v>testuser445</v>
+      </c>
+      <c r="E10" t="str">
+        <v>MPC-7006</v>
+      </c>
+      <c r="F10" t="str">
+        <v>—</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Hashed (scrypt + salt)</v>
+      </c>
+      <c r="H10" t="str">
+        <v>testuser445</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>p009</v>
+      </c>
+      <c r="B11" t="str">
+        <v>API Tester</v>
+      </c>
+      <c r="C11" t="str">
+        <v>passenger</v>
+      </c>
+      <c r="D11" t="str">
+        <v>testuser1825</v>
+      </c>
+      <c r="E11" t="str">
+        <v>MPC-7007</v>
+      </c>
+      <c r="F11" t="str">
+        <v>—</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Hashed (scrypt + salt)</v>
+      </c>
+      <c r="H11" t="str">
+        <v>testuser1825</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>p010</v>
+      </c>
+      <c r="B12" t="str">
+        <v>API Tester</v>
+      </c>
+      <c r="C12" t="str">
+        <v>passenger</v>
+      </c>
+      <c r="D12" t="str">
+        <v>testuser8302</v>
+      </c>
+      <c r="E12" t="str">
+        <v>MPC-7008</v>
+      </c>
+      <c r="F12" t="str">
+        <v>—</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Hashed (scrypt + salt)</v>
+      </c>
+      <c r="H12" t="str">
+        <v>testuser8302</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement journey planner component and add backend data and routing support
</commit_message>
<xml_diff>
--- a/backend/data/users_export.xlsx
+++ b/backend/data/users_export.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H12"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -643,9 +643,87 @@
         <v>testuser2782</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>p008</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Test User</v>
+      </c>
+      <c r="C10" t="str">
+        <v>passenger</v>
+      </c>
+      <c r="D10" t="str">
+        <v>user_test_999</v>
+      </c>
+      <c r="E10" t="str">
+        <v>MPC-7006</v>
+      </c>
+      <c r="F10" t="str">
+        <v>—</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Hashed (scrypt + salt)</v>
+      </c>
+      <c r="H10" t="str">
+        <v>user_test_999</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>p009</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Taufique Shaikh</v>
+      </c>
+      <c r="C11" t="str">
+        <v>passenger</v>
+      </c>
+      <c r="D11" t="str">
+        <v>taufique.shaikh@theemcoe.org</v>
+      </c>
+      <c r="E11" t="str">
+        <v>MPC-7007</v>
+      </c>
+      <c r="F11" t="str">
+        <v>—</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Hashed (scrypt + salt)</v>
+      </c>
+      <c r="H11" t="str">
+        <v>taufique.shaikh@theemcoe.org</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>p010</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Test User</v>
+      </c>
+      <c r="C12" t="str">
+        <v>passenger</v>
+      </c>
+      <c r="D12" t="str">
+        <v>testuser001</v>
+      </c>
+      <c r="E12" t="str">
+        <v>MPC-7008</v>
+      </c>
+      <c r="F12" t="str">
+        <v>—</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Hashed (scrypt + salt)</v>
+      </c>
+      <c r="H12" t="str">
+        <v>testuser001</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>